<commit_message>
sync time course scripts
</commit_message>
<xml_diff>
--- a/mri-data/roi-time-courses/roi02c_stats_glm001_onset_O3_4to10.xlsx
+++ b/mri-data/roi-time-courses/roi02c_stats_glm001_onset_O3_4to10.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="56" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="126" uniqueCount="14">
   <si>
     <t>REG</t>
   </si>
@@ -107,11 +107,11 @@
     <col min="1" max="1" width="11.5703125" customWidth="true"/>
     <col min="2" max="2" width="17.85546875" customWidth="true"/>
     <col min="3" max="3" width="21.85546875" customWidth="true"/>
-    <col min="4" max="4" width="12.42578125" customWidth="true"/>
+    <col min="4" max="4" width="14.42578125" customWidth="true"/>
     <col min="5" max="5" width="12.7109375" customWidth="true"/>
     <col min="6" max="6" width="12.42578125" customWidth="true"/>
     <col min="7" max="7" width="5.42578125" customWidth="true"/>
-    <col min="8" max="8" width="14.7109375" customWidth="true"/>
+    <col min="8" max="8" width="15.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -151,19 +151,19 @@
         <v>6</v>
       </c>
       <c r="D2" s="0">
-        <v>-0.47755698503279009</v>
+        <v>-0.073041061863310955</v>
       </c>
       <c r="E2" s="0">
-        <v>0.74880859190454396</v>
+        <v>0.10723497846384428</v>
       </c>
       <c r="F2" s="0">
-        <v>-3.5508737362686018</v>
+        <v>-3.7923765835689687</v>
       </c>
       <c r="G2" s="0">
         <v>30</v>
       </c>
       <c r="H2" s="0">
-        <v>0.0012898405724040872</v>
+        <v>0.00067335400913862121</v>
       </c>
     </row>
     <row r="3">
@@ -177,19 +177,19 @@
         <v>7</v>
       </c>
       <c r="D3" s="0">
-        <v>0.19331160064221389</v>
+        <v>0.045956608393245099</v>
       </c>
       <c r="E3" s="0">
-        <v>0.97499797833137059</v>
+        <v>0.15147770256889911</v>
       </c>
       <c r="F3" s="0">
-        <v>1.1039135104868323</v>
+        <v>1.6891962454478144</v>
       </c>
       <c r="G3" s="0">
         <v>30</v>
       </c>
       <c r="H3" s="0">
-        <v>0.27840680433799569</v>
+        <v>0.10155060964299779</v>
       </c>
     </row>
   </sheetData>
@@ -208,7 +208,7 @@
     <col min="5" max="5" width="12.7109375" customWidth="true"/>
     <col min="6" max="6" width="11.7109375" customWidth="true"/>
     <col min="7" max="7" width="5.42578125" customWidth="true"/>
-    <col min="8" max="8" width="13.7109375" customWidth="true"/>
+    <col min="8" max="8" width="12.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -248,19 +248,19 @@
         <v>6</v>
       </c>
       <c r="D2" s="0">
-        <v>0.057595987728165023</v>
+        <v>0.058414789561025839</v>
       </c>
       <c r="E2" s="0">
-        <v>0.14015042630389923</v>
+        <v>0.13924334181449721</v>
       </c>
       <c r="F2" s="0">
-        <v>2.2881192470975065</v>
+        <v>2.3357654257780296</v>
       </c>
       <c r="G2" s="0">
         <v>30</v>
       </c>
       <c r="H2" s="0">
-        <v>0.029349032938800323</v>
+        <v>0.026378910399511978</v>
       </c>
     </row>
     <row r="3">
@@ -274,19 +274,19 @@
         <v>7</v>
       </c>
       <c r="D3" s="0">
-        <v>-0.02537764748933511</v>
+        <v>-0.02595019485942467</v>
       </c>
       <c r="E3" s="0">
-        <v>0.14703250723446099</v>
+        <v>0.14678905114669749</v>
       </c>
       <c r="F3" s="0">
-        <v>-0.96098994678957728</v>
+        <v>-0.98430072963960402</v>
       </c>
       <c r="G3" s="0">
         <v>30</v>
       </c>
       <c r="H3" s="0">
-        <v>0.34423926729056276</v>
+        <v>0.33283993399738354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>